<commit_message>
added more test cases in LearnLocators spec file
</commit_message>
<xml_diff>
--- a/tests2/Anvesh.xlsx
+++ b/tests2/Anvesh.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/369c40edd623e24e/Documents/PlaywrightDemo/PlaywrightDemo/tests2/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AnandaBabuGummadilli\Documents\Anand_Details\Training\PlaywrightDemo\tests2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="8_{4C6BB314-4BFC-44AE-BD4F-A654D6C3D3AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3D4A4780-723A-4718-A627-5AAE7465D9E0}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CD7444D-2C16-44CD-9559-BDAF0F4F18E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{147B6599-C5F3-4C20-9670-D864EFFB2C93}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{147B6599-C5F3-4C20-9670-D864EFFB2C93}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,9 +36,36 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
-  <si>
-    <t>asha</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+  <si>
+    <t>Anvesh</t>
+  </si>
+  <si>
+    <t>Hyderabad</t>
+  </si>
+  <si>
+    <t>Asha</t>
+  </si>
+  <si>
+    <t>Beeramguda</t>
+  </si>
+  <si>
+    <t>Anand</t>
+  </si>
+  <si>
+    <t>Bangalore</t>
+  </si>
+  <si>
+    <t>Mike</t>
+  </si>
+  <si>
+    <t>Dallas</t>
+  </si>
+  <si>
+    <t>Steve</t>
+  </si>
+  <si>
+    <t>Irving</t>
   </si>
 </sst>
 </file>
@@ -417,13 +444,51 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57C6250A-37D1-42EF-9B6D-0A2375BA4B66}">
-  <dimension ref="B11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="11" spans="2:2" ht="15" x14ac:dyDescent="0.3">
-      <c r="B11" s="1" t="s">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="16" x14ac:dyDescent="0.4">
+      <c r="B11" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>